<commit_message>
run for 2020-2024 for insights 2025 update
</commit_message>
<xml_diff>
--- a/output_data/charts/crashSeverityByType-Delaware.xlsx
+++ b/output_data/charts/crashSeverityByType-Delaware.xlsx
@@ -40,43 +40,43 @@
     <t>Sideswipe - Passing</t>
   </si>
   <si>
+    <t>Pedestrian</t>
+  </si>
+  <si>
+    <t>Left Turn</t>
+  </si>
+  <si>
     <t>Rear End</t>
   </si>
   <si>
-    <t>Pedestrian</t>
+    <t>Overturning</t>
+  </si>
+  <si>
+    <t>Parked Vehicle</t>
+  </si>
+  <si>
+    <t>Right Turn</t>
+  </si>
+  <si>
+    <t>Animal</t>
   </si>
   <si>
     <t>Pedalcycles</t>
   </si>
   <si>
-    <t>Left Turn</t>
-  </si>
-  <si>
-    <t>Right Turn</t>
-  </si>
-  <si>
-    <t>Parked Vehicle</t>
+    <t>Other Object</t>
+  </si>
+  <si>
+    <t>Other Non-Collision</t>
+  </si>
+  <si>
+    <t>Sideswipe - Meeting</t>
+  </si>
+  <si>
+    <t>Backing</t>
   </si>
   <si>
     <t>Train</t>
-  </si>
-  <si>
-    <t>Sideswipe - Meeting</t>
-  </si>
-  <si>
-    <t>Animal</t>
-  </si>
-  <si>
-    <t>Backing</t>
-  </si>
-  <si>
-    <t>Overturning</t>
-  </si>
-  <si>
-    <t>Other Object</t>
-  </si>
-  <si>
-    <t>Other Non-Collision</t>
   </si>
   <si>
     <t>Unknown</t>
@@ -228,43 +228,43 @@
                   <c:v>Sideswipe - Passing</c:v>
                 </c:pt>
                 <c:pt idx="4">
+                  <c:v>Pedestrian</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>Left Turn</c:v>
+                </c:pt>
+                <c:pt idx="6">
                   <c:v>Rear End</c:v>
                 </c:pt>
-                <c:pt idx="5">
-                  <c:v>Pedestrian</c:v>
-                </c:pt>
-                <c:pt idx="6">
+                <c:pt idx="7">
+                  <c:v>Overturning</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>Parked Vehicle</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>Right Turn</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>Animal</c:v>
+                </c:pt>
+                <c:pt idx="11">
                   <c:v>Pedalcycles</c:v>
                 </c:pt>
-                <c:pt idx="7">
-                  <c:v>Left Turn</c:v>
-                </c:pt>
-                <c:pt idx="8">
-                  <c:v>Right Turn</c:v>
-                </c:pt>
-                <c:pt idx="9">
-                  <c:v>Parked Vehicle</c:v>
-                </c:pt>
-                <c:pt idx="10">
+                <c:pt idx="12">
+                  <c:v>Other Object</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>Other Non-Collision</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>Sideswipe - Meeting</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>Backing</c:v>
+                </c:pt>
+                <c:pt idx="16">
                   <c:v>Train</c:v>
-                </c:pt>
-                <c:pt idx="11">
-                  <c:v>Sideswipe - Meeting</c:v>
-                </c:pt>
-                <c:pt idx="12">
-                  <c:v>Animal</c:v>
-                </c:pt>
-                <c:pt idx="13">
-                  <c:v>Backing</c:v>
-                </c:pt>
-                <c:pt idx="14">
-                  <c:v>Overturning</c:v>
-                </c:pt>
-                <c:pt idx="15">
-                  <c:v>Other Object</c:v>
-                </c:pt>
-                <c:pt idx="16">
-                  <c:v>Other Non-Collision</c:v>
                 </c:pt>
                 <c:pt idx="17">
                   <c:v>Unknown</c:v>
@@ -279,40 +279,40 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="18"/>
                 <c:pt idx="0">
-                  <c:v>33.33333333333333</c:v>
+                  <c:v>29.33333333333333</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>17.39130434782609</c:v>
+                  <c:v>20</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>13.04347826086956</c:v>
+                  <c:v>18.66666666666667</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>8.695652173913043</c:v>
+                  <c:v>8</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>7.246376811594203</c:v>
+                  <c:v>6.666666666666667</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>7.246376811594203</c:v>
+                  <c:v>5.333333333333334</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>4.347826086956522</c:v>
+                  <c:v>5.333333333333334</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>2.898550724637681</c:v>
+                  <c:v>2.666666666666667</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>1.449275362318841</c:v>
+                  <c:v>2.666666666666667</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>1.449275362318841</c:v>
+                  <c:v>1.333333333333333</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>1.449275362318841</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>1.449275362318841</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="12">
                   <c:v>0</c:v>
@@ -376,43 +376,43 @@
                   <c:v>Sideswipe - Passing</c:v>
                 </c:pt>
                 <c:pt idx="4">
+                  <c:v>Pedestrian</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>Left Turn</c:v>
+                </c:pt>
+                <c:pt idx="6">
                   <c:v>Rear End</c:v>
                 </c:pt>
-                <c:pt idx="5">
-                  <c:v>Pedestrian</c:v>
-                </c:pt>
-                <c:pt idx="6">
+                <c:pt idx="7">
+                  <c:v>Overturning</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>Parked Vehicle</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>Right Turn</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>Animal</c:v>
+                </c:pt>
+                <c:pt idx="11">
                   <c:v>Pedalcycles</c:v>
                 </c:pt>
-                <c:pt idx="7">
-                  <c:v>Left Turn</c:v>
-                </c:pt>
-                <c:pt idx="8">
-                  <c:v>Right Turn</c:v>
-                </c:pt>
-                <c:pt idx="9">
-                  <c:v>Parked Vehicle</c:v>
-                </c:pt>
-                <c:pt idx="10">
+                <c:pt idx="12">
+                  <c:v>Other Object</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>Other Non-Collision</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>Sideswipe - Meeting</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>Backing</c:v>
+                </c:pt>
+                <c:pt idx="16">
                   <c:v>Train</c:v>
-                </c:pt>
-                <c:pt idx="11">
-                  <c:v>Sideswipe - Meeting</c:v>
-                </c:pt>
-                <c:pt idx="12">
-                  <c:v>Animal</c:v>
-                </c:pt>
-                <c:pt idx="13">
-                  <c:v>Backing</c:v>
-                </c:pt>
-                <c:pt idx="14">
-                  <c:v>Overturning</c:v>
-                </c:pt>
-                <c:pt idx="15">
-                  <c:v>Other Object</c:v>
-                </c:pt>
-                <c:pt idx="16">
-                  <c:v>Other Non-Collision</c:v>
                 </c:pt>
                 <c:pt idx="17">
                   <c:v>Unknown</c:v>
@@ -427,55 +427,55 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="18"/>
                 <c:pt idx="0">
-                  <c:v>22.05513784461153</c:v>
+                  <c:v>20.14051522248243</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>25.31328320802005</c:v>
+                  <c:v>27.16627634660422</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>6.516290726817042</c:v>
+                  <c:v>7.728337236533958</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>4.511278195488721</c:v>
+                  <c:v>5.85480093676815</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>9.523809523809524</c:v>
+                  <c:v>4.683840749414521</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>5.263157894736842</c:v>
+                  <c:v>12.88056206088993</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>4.260651629072681</c:v>
+                  <c:v>9.601873536299765</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>13.7844611528822</c:v>
+                  <c:v>4.449648711943794</c:v>
                 </c:pt>
                 <c:pt idx="8">
+                  <c:v>1.639344262295082</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>0.468384074941452</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>1.639344262295082</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>3.044496487119438</c:v>
+                </c:pt>
+                <c:pt idx="12">
                   <c:v>0</c:v>
                 </c:pt>
-                <c:pt idx="9">
-                  <c:v>2.005012531328321</c:v>
-                </c:pt>
-                <c:pt idx="10">
+                <c:pt idx="13">
+                  <c:v>0.702576112412178</c:v>
+                </c:pt>
+                <c:pt idx="14">
                   <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="11">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="12">
-                  <c:v>1.754385964912281</c:v>
-                </c:pt>
-                <c:pt idx="13">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="14">
-                  <c:v>4.511278195488721</c:v>
                 </c:pt>
                 <c:pt idx="15">
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="16">
-                  <c:v>0.5012531328320802</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="17">
                   <c:v>0</c:v>
@@ -524,43 +524,43 @@
                   <c:v>Sideswipe - Passing</c:v>
                 </c:pt>
                 <c:pt idx="4">
+                  <c:v>Pedestrian</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>Left Turn</c:v>
+                </c:pt>
+                <c:pt idx="6">
                   <c:v>Rear End</c:v>
                 </c:pt>
-                <c:pt idx="5">
-                  <c:v>Pedestrian</c:v>
-                </c:pt>
-                <c:pt idx="6">
+                <c:pt idx="7">
+                  <c:v>Overturning</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>Parked Vehicle</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>Right Turn</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>Animal</c:v>
+                </c:pt>
+                <c:pt idx="11">
                   <c:v>Pedalcycles</c:v>
                 </c:pt>
-                <c:pt idx="7">
-                  <c:v>Left Turn</c:v>
-                </c:pt>
-                <c:pt idx="8">
-                  <c:v>Right Turn</c:v>
-                </c:pt>
-                <c:pt idx="9">
-                  <c:v>Parked Vehicle</c:v>
-                </c:pt>
-                <c:pt idx="10">
+                <c:pt idx="12">
+                  <c:v>Other Object</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>Other Non-Collision</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>Sideswipe - Meeting</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>Backing</c:v>
+                </c:pt>
+                <c:pt idx="16">
                   <c:v>Train</c:v>
-                </c:pt>
-                <c:pt idx="11">
-                  <c:v>Sideswipe - Meeting</c:v>
-                </c:pt>
-                <c:pt idx="12">
-                  <c:v>Animal</c:v>
-                </c:pt>
-                <c:pt idx="13">
-                  <c:v>Backing</c:v>
-                </c:pt>
-                <c:pt idx="14">
-                  <c:v>Overturning</c:v>
-                </c:pt>
-                <c:pt idx="15">
-                  <c:v>Other Object</c:v>
-                </c:pt>
-                <c:pt idx="16">
-                  <c:v>Other Non-Collision</c:v>
                 </c:pt>
                 <c:pt idx="17">
                   <c:v>Unknown</c:v>
@@ -575,58 +575,58 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="18"/>
                 <c:pt idx="0">
-                  <c:v>15.91758179553945</c:v>
+                  <c:v>15.57588552662444</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>12.95709272048002</c:v>
+                  <c:v>13.66408632418485</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>1.692516698743349</c:v>
+                  <c:v>1.788646493079991</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>10.97588588248613</c:v>
+                  <c:v>11.02509969505043</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>28.02558587116495</c:v>
+                  <c:v>0.6509500351864884</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>0.6622891429865277</c:v>
+                  <c:v>7.095941825005865</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>0.4924714140156232</c:v>
+                  <c:v>26.93525686136524</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>6.656854975659458</c:v>
+                  <c:v>0.6685432793807178</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>2.768028982225744</c:v>
+                  <c:v>3.794276331222144</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>3.600135854183176</c:v>
+                  <c:v>2.785596997419657</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>0.01698177289709046</c:v>
+                  <c:v>9.459300961764015</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>0.12453300124533</c:v>
+                  <c:v>0.4867464227070138</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>9.453186912713688</c:v>
+                  <c:v>0.5688482289467511</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>3.311445714932639</c:v>
+                  <c:v>1.477832512315271</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>0.6283255971923468</c:v>
+                  <c:v>0.09383063570255688</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>0.594362051398166</c:v>
+                  <c:v>3.266479005395261</c:v>
                 </c:pt>
                 <c:pt idx="16">
-                  <c:v>1.528359560738141</c:v>
+                  <c:v>0.01172882946281961</c:v>
                 </c:pt>
                 <c:pt idx="17">
-                  <c:v>0.594362051398166</c:v>
+                  <c:v>0.6509500351864884</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1082,13 +1082,13 @@
         <v>4</v>
       </c>
       <c r="B2" s="2">
-        <v>33.33333333333333</v>
+        <v>29.33333333333333</v>
       </c>
       <c r="C2" s="2">
-        <v>22.05513784461153</v>
+        <v>20.14051522248243</v>
       </c>
       <c r="D2" s="2">
-        <v>15.91758179553945</v>
+        <v>15.57588552662444</v>
       </c>
     </row>
     <row r="3" spans="1:4">
@@ -1096,13 +1096,13 @@
         <v>5</v>
       </c>
       <c r="B3" s="2">
-        <v>17.39130434782609</v>
+        <v>20</v>
       </c>
       <c r="C3" s="2">
-        <v>25.31328320802005</v>
+        <v>27.16627634660422</v>
       </c>
       <c r="D3" s="2">
-        <v>12.95709272048002</v>
+        <v>13.66408632418485</v>
       </c>
     </row>
     <row r="4" spans="1:4">
@@ -1110,13 +1110,13 @@
         <v>6</v>
       </c>
       <c r="B4" s="2">
-        <v>13.04347826086956</v>
+        <v>18.66666666666667</v>
       </c>
       <c r="C4" s="2">
-        <v>6.516290726817042</v>
+        <v>7.728337236533958</v>
       </c>
       <c r="D4" s="2">
-        <v>1.692516698743349</v>
+        <v>1.788646493079991</v>
       </c>
     </row>
     <row r="5" spans="1:4">
@@ -1124,13 +1124,13 @@
         <v>7</v>
       </c>
       <c r="B5" s="2">
-        <v>8.695652173913043</v>
+        <v>8</v>
       </c>
       <c r="C5" s="2">
-        <v>4.511278195488721</v>
+        <v>5.85480093676815</v>
       </c>
       <c r="D5" s="2">
-        <v>10.97588588248613</v>
+        <v>11.02509969505043</v>
       </c>
     </row>
     <row r="6" spans="1:4">
@@ -1138,13 +1138,13 @@
         <v>8</v>
       </c>
       <c r="B6" s="2">
-        <v>7.246376811594203</v>
+        <v>6.666666666666667</v>
       </c>
       <c r="C6" s="2">
-        <v>9.523809523809524</v>
+        <v>4.683840749414521</v>
       </c>
       <c r="D6" s="2">
-        <v>28.02558587116495</v>
+        <v>0.6509500351864884</v>
       </c>
     </row>
     <row r="7" spans="1:4">
@@ -1152,13 +1152,13 @@
         <v>9</v>
       </c>
       <c r="B7" s="2">
-        <v>7.246376811594203</v>
+        <v>5.333333333333334</v>
       </c>
       <c r="C7" s="2">
-        <v>5.263157894736842</v>
+        <v>12.88056206088993</v>
       </c>
       <c r="D7" s="2">
-        <v>0.6622891429865277</v>
+        <v>7.095941825005865</v>
       </c>
     </row>
     <row r="8" spans="1:4">
@@ -1166,13 +1166,13 @@
         <v>10</v>
       </c>
       <c r="B8" s="2">
-        <v>4.347826086956522</v>
+        <v>5.333333333333334</v>
       </c>
       <c r="C8" s="2">
-        <v>4.260651629072681</v>
+        <v>9.601873536299765</v>
       </c>
       <c r="D8" s="2">
-        <v>0.4924714140156232</v>
+        <v>26.93525686136524</v>
       </c>
     </row>
     <row r="9" spans="1:4">
@@ -1180,13 +1180,13 @@
         <v>11</v>
       </c>
       <c r="B9" s="2">
-        <v>2.898550724637681</v>
+        <v>2.666666666666667</v>
       </c>
       <c r="C9" s="2">
-        <v>13.7844611528822</v>
+        <v>4.449648711943794</v>
       </c>
       <c r="D9" s="2">
-        <v>6.656854975659458</v>
+        <v>0.6685432793807178</v>
       </c>
     </row>
     <row r="10" spans="1:4">
@@ -1194,13 +1194,13 @@
         <v>12</v>
       </c>
       <c r="B10" s="2">
-        <v>1.449275362318841</v>
+        <v>2.666666666666667</v>
       </c>
       <c r="C10" s="2">
-        <v>0</v>
+        <v>1.639344262295082</v>
       </c>
       <c r="D10" s="2">
-        <v>2.768028982225744</v>
+        <v>3.794276331222144</v>
       </c>
     </row>
     <row r="11" spans="1:4">
@@ -1208,13 +1208,13 @@
         <v>13</v>
       </c>
       <c r="B11" s="2">
-        <v>1.449275362318841</v>
+        <v>1.333333333333333</v>
       </c>
       <c r="C11" s="2">
-        <v>2.005012531328321</v>
+        <v>0.468384074941452</v>
       </c>
       <c r="D11" s="2">
-        <v>3.600135854183176</v>
+        <v>2.785596997419657</v>
       </c>
     </row>
     <row r="12" spans="1:4">
@@ -1222,13 +1222,13 @@
         <v>14</v>
       </c>
       <c r="B12" s="2">
-        <v>1.449275362318841</v>
+        <v>0</v>
       </c>
       <c r="C12" s="2">
-        <v>0</v>
+        <v>1.639344262295082</v>
       </c>
       <c r="D12" s="2">
-        <v>0.01698177289709046</v>
+        <v>9.459300961764015</v>
       </c>
     </row>
     <row r="13" spans="1:4">
@@ -1236,13 +1236,13 @@
         <v>15</v>
       </c>
       <c r="B13" s="2">
-        <v>1.449275362318841</v>
+        <v>0</v>
       </c>
       <c r="C13" s="2">
-        <v>0</v>
+        <v>3.044496487119438</v>
       </c>
       <c r="D13" s="2">
-        <v>0.12453300124533</v>
+        <v>0.4867464227070138</v>
       </c>
     </row>
     <row r="14" spans="1:4">
@@ -1253,10 +1253,10 @@
         <v>0</v>
       </c>
       <c r="C14" s="2">
-        <v>1.754385964912281</v>
+        <v>0</v>
       </c>
       <c r="D14" s="2">
-        <v>9.453186912713688</v>
+        <v>0.5688482289467511</v>
       </c>
     </row>
     <row r="15" spans="1:4">
@@ -1267,10 +1267,10 @@
         <v>0</v>
       </c>
       <c r="C15" s="2">
-        <v>0</v>
+        <v>0.702576112412178</v>
       </c>
       <c r="D15" s="2">
-        <v>3.311445714932639</v>
+        <v>1.477832512315271</v>
       </c>
     </row>
     <row r="16" spans="1:4">
@@ -1281,10 +1281,10 @@
         <v>0</v>
       </c>
       <c r="C16" s="2">
-        <v>4.511278195488721</v>
+        <v>0</v>
       </c>
       <c r="D16" s="2">
-        <v>0.6283255971923468</v>
+        <v>0.09383063570255688</v>
       </c>
     </row>
     <row r="17" spans="1:4">
@@ -1298,7 +1298,7 @@
         <v>0</v>
       </c>
       <c r="D17" s="2">
-        <v>0.594362051398166</v>
+        <v>3.266479005395261</v>
       </c>
     </row>
     <row r="18" spans="1:4">
@@ -1309,10 +1309,10 @@
         <v>0</v>
       </c>
       <c r="C18" s="2">
-        <v>0.5012531328320802</v>
+        <v>0</v>
       </c>
       <c r="D18" s="2">
-        <v>1.528359560738141</v>
+        <v>0.01172882946281961</v>
       </c>
     </row>
     <row r="19" spans="1:4">
@@ -1326,7 +1326,7 @@
         <v>0</v>
       </c>
       <c r="D19" s="2">
-        <v>0.594362051398166</v>
+        <v>0.6509500351864884</v>
       </c>
     </row>
   </sheetData>

</xml_diff>